<commit_message>
feat: add sample data
</commit_message>
<xml_diff>
--- a/templates/www.teseu.net_template.xlsx
+++ b/templates/www.teseu.net_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias/EliasLi/03.code-github/formfiller-excel-chrome/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D9BCC8-B183-9D4A-9690-F840937847F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EFE9511-B567-4D4B-ADAA-CEF8CBCE07EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4280" yWindow="2620" windowWidth="24780" windowHeight="16700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>名字</t>
   </si>
@@ -55,9 +55,6 @@
     <t>标题</t>
   </si>
   <si>
-    <t>ambrose.john@163.com</t>
-  </si>
-  <si>
     <t>独立站链接</t>
   </si>
   <si>
@@ -66,12 +63,27 @@
   <si>
     <t>great</t>
   </si>
+  <si>
+    <t>ambrose.john@gmail.com</t>
+  </si>
+  <si>
+    <t>ken.chui@gmail.com</t>
+  </si>
+  <si>
+    <t>Ken Chui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">great </t>
+  </si>
+  <si>
+    <t>https://www.teseu.net/shop/teseu-glp-1-patches-weight-management-blue/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,6 +159,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -173,7 +192,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -198,6 +217,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -744,7 +766,7 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
@@ -758,24 +780,37 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="C3" s="8"/>
-      <c r="E3" s="3"/>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="C4" s="8"/>
@@ -7196,66 +7231,67 @@
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="C1731:C1048576 C1">
-    <cfRule type="duplicateValues" dxfId="25" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="73"/>
+  <conditionalFormatting sqref="A2:A3">
+    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C8">
-    <cfRule type="duplicateValues" dxfId="22" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+  <conditionalFormatting sqref="C2:C3">
+    <cfRule type="duplicateValues" dxfId="22" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="87"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C8">
+    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9:C214 C226:C238 C248:C258 C1050:C1397 C534:C778 C437:C511">
-    <cfRule type="duplicateValues" dxfId="19" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9:C511 C534:C778 C1050:C1397">
-    <cfRule type="duplicateValues" dxfId="18" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9:C1730">
-    <cfRule type="duplicateValues" dxfId="17" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C77:C82 C87:C107 C59:C74 C55:C57 C29:C52 C15:C23 C9:C11">
-    <cfRule type="duplicateValues" dxfId="16" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C259 C261:C272">
-    <cfRule type="duplicateValues" dxfId="13" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C273:C301">
-    <cfRule type="duplicateValues" dxfId="12" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C322:C326 C356:C359 C371 C374:C376 C361:C369 C344:C353 C328:C342">
-    <cfRule type="duplicateValues" dxfId="11" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C512:C531">
-    <cfRule type="duplicateValues" dxfId="10" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C814:C824 C826:C855 C976:C1001 C962:C969 C956:C960 C884:C954 C971:C974 C875:C882 C1007:C1016 C1018:C1022 C1024:C1042 C779:C788 C1003:C1005 C810:C812 C794:C808 C857:C873 C790:C792">
-    <cfRule type="duplicateValues" dxfId="9" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1398:C1435">
-    <cfRule type="duplicateValues" dxfId="8" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1451:C1454 C1456:C1459 C1461:C1465 C1479 C1481 C1483:C1487 C1489:C1491 C1493:C1495 C1508:C1509 C1511:C1521 C1524 C1530 C1532 C1538:C1555 C1526:C1528 C1557:C1576 C1502:C1505 C1497:C1500 C1468:C1477">
-    <cfRule type="duplicateValues" dxfId="7" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1585:C1591 C1601:C1621 C1594:C1598 C1577:C1582 C1665 C1645:C1663 C1632:C1642 C1623:C1630">
-    <cfRule type="duplicateValues" dxfId="6" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="49"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2">
-    <cfRule type="duplicateValues" dxfId="5" priority="86"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="87"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="88"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  <conditionalFormatting sqref="C1731:C1048576 C1">
+    <cfRule type="duplicateValues" dxfId="2" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="73"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{78433328-95A1-40F6-B009-D5E87C666903}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{98FD3B61-B8E3-9941-8A12-F647B7304927}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>